<commit_message>
Complete Sprint 2 MFA flow and refactor database access
</commit_message>
<xml_diff>
--- a/docs/test-cases/SmartBank_US001_Complete_QA_Test_Plan.xlsx
+++ b/docs/test-cases/SmartBank_US001_Complete_QA_Test_Plan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pl_ba\PycharmProjects\MyTestProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pl_ba\PycharmProjects\MyTestProject\smartbank-qa-automation\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0D9225-C521-49AF-8FC9-7BEE5BAFC2F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD283748-92E6-44B9-A09F-78B025B16432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="US -001. QA Test Cases" sheetId="1" r:id="rId1"/>

</xml_diff>